<commit_message>
Adjust benchmarking to avoid unrecognized images
Signed-off-by: Willian Rampazzo <w095284@dac.unicamp.br>
</commit_message>
<xml_diff>
--- a/projects/ed-xai/reports/benchmark/benchmark.xlsx
+++ b/projects/ed-xai/reports/benchmark/benchmark.xlsx
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0.9912</v>
+        <v>0.9892</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.9878</v>
+        <v>0.985</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>0.5706</v>
@@ -554,10 +554,10 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.99</v>
+        <v>0.9898</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.9861</v>
+        <v>0.9859</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>0.5712</v>

</xml_diff>